<commit_message>
Update README.md with project description
</commit_message>
<xml_diff>
--- a/testCases/Lereve Manual Testing.xlsx
+++ b/testCases/Lereve Manual Testing.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="78">
   <si>
     <t>Please click here to see the full  pdf</t>
   </si>
@@ -170,7 +170,13 @@
     <t>Final Status</t>
   </si>
   <si>
+    <t>Header Module</t>
+  </si>
+  <si>
     <t>UI Testing</t>
+  </si>
+  <si>
+    <t>Header Section</t>
   </si>
   <si>
     <t>Verify header section is displayed on the website</t>
@@ -187,6 +193,66 @@
   </si>
   <si>
     <t>Passed</t>
+  </si>
+  <si>
+    <t>Header
+ Alignment</t>
+  </si>
+  <si>
+    <t>Logo Alignment</t>
+  </si>
+  <si>
+    <t>Header 
+Consistency</t>
+  </si>
+  <si>
+    <t>Icons &amp; Text</t>
+  </si>
+  <si>
+    <t>Dropdown Menu</t>
+  </si>
+  <si>
+    <t>Not found as per as 
+expectation</t>
+  </si>
+  <si>
+    <t>Functional 
+Testing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header Links
+</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Logo Navigation</t>
+  </si>
+  <si>
+    <t>Search Bar</t>
+  </si>
+  <si>
+    <t>Search Module</t>
+  </si>
+  <si>
+    <t>Search Field</t>
+  </si>
+  <si>
+    <t>Verify spelling and grammar 
+of placeholder</t>
+  </si>
+  <si>
+    <t>Text should be correct</t>
+  </si>
+  <si>
+    <t>Found as per as expectations</t>
+  </si>
+  <si>
+    <t>Oprn Page</t>
+  </si>
+  <si>
+    <t>Search Icon</t>
   </si>
   <si>
     <t>t</t>
@@ -199,7 +265,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -252,6 +318,20 @@
     </font>
     <font>
       <b/>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -350,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -410,10 +490,16 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -424,6 +510,18 @@
     </xf>
     <xf borderId="0" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -887,8 +985,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="5" max="5" width="13.25"/>
-    <col customWidth="1" min="7" max="7" width="15.38"/>
+    <col customWidth="1" min="4" max="4" width="22.13"/>
+    <col customWidth="1" min="5" max="5" width="19.5"/>
+    <col customWidth="1" min="6" max="6" width="22.88"/>
+    <col customWidth="1" min="7" max="7" width="17.63"/>
     <col customWidth="1" min="8" max="8" width="13.88"/>
   </cols>
   <sheetData>
@@ -962,51 +1062,193 @@
       <c r="Y5" s="20"/>
       <c r="Z5" s="20"/>
     </row>
-    <row r="6">
-      <c r="A6" s="21">
+    <row r="6" ht="31.5" customHeight="1">
+      <c r="A6" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="22"/>
+      <c r="Z6" s="22"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23">
         <v>1.0</v>
       </c>
-      <c r="B6" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="23" t="s">
+      <c r="B7" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="C7" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="D7" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="E7" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="H6" s="20"/>
-      <c r="I6" s="25" t="s">
+      <c r="F7" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
-      <c r="T6" s="20"/>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
-      <c r="W6" s="20"/>
-      <c r="X6" s="20"/>
-      <c r="Y6" s="20"/>
-      <c r="Z6" s="20"/>
-    </row>
+      <c r="G7" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="20"/>
+      <c r="I7" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
+      <c r="X7" s="20"/>
+      <c r="Y7" s="20"/>
+      <c r="Z7" s="20"/>
+    </row>
+    <row r="8" ht="48.75" customHeight="1">
+      <c r="A8" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" ht="47.25" customHeight="1">
+      <c r="A9" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" ht="49.5" customHeight="1">
+      <c r="A10" s="9">
+        <v>4.0</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" ht="54.0" customHeight="1">
+      <c r="A11" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" ht="52.5" customHeight="1">
+      <c r="A12" s="9">
+        <v>6.0</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" ht="46.5" customHeight="1">
+      <c r="B13" s="29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" ht="51.75" customHeight="1">
+      <c r="A14" s="9">
+        <v>7.0</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" ht="60.0" customHeight="1">
+      <c r="A15" s="9">
+        <v>8.0</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" ht="52.5" customHeight="1">
+      <c r="A16" s="9">
+        <v>9.0</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" ht="52.5" customHeight="1">
+      <c r="A17" s="9">
+        <v>10.0</v>
+      </c>
+      <c r="C17" s="29" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" ht="52.5" customHeight="1">
+      <c r="A18" s="30" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" ht="52.5" customHeight="1">
+      <c r="B19" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" ht="52.5" customHeight="1">
+      <c r="C20" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" ht="52.5" customHeight="1">
+      <c r="C21" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" ht="52.5" customHeight="1"/>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A18:I18"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B1"/>
   </hyperlinks>
@@ -1023,7 +1265,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>